<commit_message>
Aggiunta sub tabs, refactoring tabelle excel e conseguente modifica del problem generator. Modifica gitignore per ignorare il file temporaanei di libre office
</commit_message>
<xml_diff>
--- a/application/GUI/xlsx/Difficulty1.xlsx
+++ b/application/GUI/xlsx/Difficulty1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="corsi" sheetId="1" state="visible" r:id="rId3"/>
@@ -26,16 +26,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="70">
   <si>
-    <t xml:space="preserve">corso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ore settimanali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">professore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gruppoStudenti</t>
+    <t xml:space="preserve">Corso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ore Settimanali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Professore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GruppoStudenti</t>
   </si>
   <si>
     <t xml:space="preserve">sistemiDigitali</t>
@@ -218,22 +218,22 @@
     <t xml:space="preserve">fri18</t>
   </si>
   <si>
-    <t xml:space="preserve">aula</t>
+    <t xml:space="preserve">Aula</t>
   </si>
   <si>
     <t xml:space="preserve">N6</t>
   </si>
   <si>
-    <t xml:space="preserve">gruppiStudenti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">configurazioni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valori</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ora pausa pranzo</t>
+    <t xml:space="preserve">GruppiStudenti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ora Pausa Pranzo</t>
   </si>
 </sst>
 </file>
@@ -338,34 +338,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -511,7 +511,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.38"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -572,7 +578,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BD3"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.68"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1101,7 +1110,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BD2"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1460,7 +1469,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BD2"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.16"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1819,7 +1831,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.89"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>